<commit_message>
Think3D repro: 3-run results for Qwen3-VL-4B and released SPAgent-4B, px256k ablation
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/think3d_repro/outputs/run1/vlmeval_runs/SPAgent_4B_no_tools_general/MindCube/SPAgent_4B_no_tools_general_MindCube.xlsx
+++ b/think3d_repro/outputs/run1/vlmeval_runs/SPAgent_4B_no_tools_general/MindCube/SPAgent_4B_no_tools_general_MindCube.xlsx
@@ -3103,7 +3103,7 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>9.69303560256958</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -3132,7 +3132,7 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>7.917886972427368</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -3161,7 +3161,7 @@
         <v>1</v>
       </c>
       <c r="I4">
-        <v>29.18851923942566</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -3190,7 +3190,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>3.860100746154785</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -3219,7 +3219,7 @@
         <v>0</v>
       </c>
       <c r="I6">
-        <v>6.236809253692627</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -3248,7 +3248,7 @@
         <v>0</v>
       </c>
       <c r="I7">
-        <v>7.822849988937378</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -3277,7 +3277,7 @@
         <v>1</v>
       </c>
       <c r="I8">
-        <v>11.36920261383057</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -3306,7 +3306,7 @@
         <v>1</v>
       </c>
       <c r="I9">
-        <v>9.660900115966797</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -3335,7 +3335,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>4.69551682472229</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -3364,7 +3364,7 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>8.265002489089966</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -3393,7 +3393,7 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>36.46648263931274</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -3422,7 +3422,7 @@
         <v>0</v>
       </c>
       <c r="I13">
-        <v>35.70666670799255</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -3451,7 +3451,7 @@
         <v>0</v>
       </c>
       <c r="I14">
-        <v>7.586764812469482</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -3480,7 +3480,7 @@
         <v>0</v>
       </c>
       <c r="I15">
-        <v>36.72700500488281</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -3509,7 +3509,7 @@
         <v>0</v>
       </c>
       <c r="I16">
-        <v>6.922994136810303</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -3538,7 +3538,7 @@
         <v>1</v>
       </c>
       <c r="I17">
-        <v>4.745076179504395</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -3567,7 +3567,7 @@
         <v>1</v>
       </c>
       <c r="I18">
-        <v>5.336412668228149</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -3596,7 +3596,7 @@
         <v>1</v>
       </c>
       <c r="I19">
-        <v>7.380324363708496</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -3625,7 +3625,7 @@
         <v>0</v>
       </c>
       <c r="I20">
-        <v>5.591073036193848</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -3654,7 +3654,7 @@
         <v>1</v>
       </c>
       <c r="I21">
-        <v>5.267738103866577</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -3683,7 +3683,7 @@
         <v>0</v>
       </c>
       <c r="I22">
-        <v>40.64112114906311</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -3712,7 +3712,7 @@
         <v>1</v>
       </c>
       <c r="I23">
-        <v>39.1012761592865</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -3741,7 +3741,7 @@
         <v>0</v>
       </c>
       <c r="I24">
-        <v>10.22247862815857</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -3770,7 +3770,7 @@
         <v>0</v>
       </c>
       <c r="I25">
-        <v>5.781538009643555</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -3799,7 +3799,7 @@
         <v>0</v>
       </c>
       <c r="I26">
-        <v>17.87110018730164</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -3828,7 +3828,7 @@
         <v>1</v>
       </c>
       <c r="I27">
-        <v>6.64234185218811</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -3857,7 +3857,7 @@
         <v>0</v>
       </c>
       <c r="I28">
-        <v>9.317964315414429</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -3886,7 +3886,7 @@
         <v>0</v>
       </c>
       <c r="I29">
-        <v>4.903970003128052</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -3915,7 +3915,7 @@
         <v>0</v>
       </c>
       <c r="I30">
-        <v>5.681869745254517</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -3944,7 +3944,7 @@
         <v>1</v>
       </c>
       <c r="I31">
-        <v>5.731046676635742</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -3973,7 +3973,7 @@
         <v>1</v>
       </c>
       <c r="I32">
-        <v>46.30612325668335</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -4002,7 +4002,7 @@
         <v>0</v>
       </c>
       <c r="I33">
-        <v>10.29637432098389</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -4031,7 +4031,7 @@
         <v>0</v>
       </c>
       <c r="I34">
-        <v>6.129546165466309</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -4060,7 +4060,7 @@
         <v>0</v>
       </c>
       <c r="I35">
-        <v>5.824615240097046</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -4089,7 +4089,7 @@
         <v>0</v>
       </c>
       <c r="I36">
-        <v>11.43218517303467</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -4118,7 +4118,7 @@
         <v>0</v>
       </c>
       <c r="I37">
-        <v>8.74774694442749</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -4147,7 +4147,7 @@
         <v>0</v>
       </c>
       <c r="I38">
-        <v>5.225991487503052</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -4176,7 +4176,7 @@
         <v>0</v>
       </c>
       <c r="I39">
-        <v>5.911834478378296</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -4205,7 +4205,7 @@
         <v>0</v>
       </c>
       <c r="I40">
-        <v>36.87946248054504</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -4234,7 +4234,7 @@
         <v>1</v>
       </c>
       <c r="I41">
-        <v>5.592250347137451</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -4263,7 +4263,7 @@
         <v>0</v>
       </c>
       <c r="I42">
-        <v>2.991460800170898</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -4292,7 +4292,7 @@
         <v>0</v>
       </c>
       <c r="I43">
-        <v>4.055252313613892</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:9">
@@ -4321,7 +4321,7 @@
         <v>1</v>
       </c>
       <c r="I44">
-        <v>5.276717901229858</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -4350,7 +4350,7 @@
         <v>1</v>
       </c>
       <c r="I45">
-        <v>2.398449182510376</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -4379,7 +4379,7 @@
         <v>1</v>
       </c>
       <c r="I46">
-        <v>5.49282431602478</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -4408,7 +4408,7 @@
         <v>1</v>
       </c>
       <c r="I47">
-        <v>2.953789710998535</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="I48">
-        <v>4.873729944229126</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -4466,7 +4466,7 @@
         <v>1</v>
       </c>
       <c r="I49">
-        <v>2.315242290496826</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -4495,7 +4495,7 @@
         <v>0</v>
       </c>
       <c r="I50">
-        <v>32.57419157028198</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -4524,7 +4524,7 @@
         <v>0</v>
       </c>
       <c r="I51">
-        <v>4.705170631408691</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -4553,7 +4553,7 @@
         <v>0</v>
       </c>
       <c r="I52">
-        <v>6.095768213272095</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -4582,7 +4582,7 @@
         <v>0</v>
       </c>
       <c r="I53">
-        <v>6.984506607055664</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -4611,7 +4611,7 @@
         <v>0</v>
       </c>
       <c r="I54">
-        <v>6.264215707778931</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -4640,7 +4640,7 @@
         <v>0</v>
       </c>
       <c r="I55">
-        <v>3.068207263946533</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -4669,7 +4669,7 @@
         <v>1</v>
       </c>
       <c r="I56">
-        <v>4.052818059921265</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:9">
@@ -4698,7 +4698,7 @@
         <v>1</v>
       </c>
       <c r="I57">
-        <v>4.449002742767334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -4727,7 +4727,7 @@
         <v>0</v>
       </c>
       <c r="I58">
-        <v>7.966551542282104</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -4756,7 +4756,7 @@
         <v>1</v>
       </c>
       <c r="I59">
-        <v>4.2254319190979</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:9">
@@ -4785,7 +4785,7 @@
         <v>0</v>
       </c>
       <c r="I60">
-        <v>4.523452520370483</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -4814,7 +4814,7 @@
         <v>0</v>
       </c>
       <c r="I61">
-        <v>3.602113485336304</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:9">
@@ -4843,7 +4843,7 @@
         <v>1</v>
       </c>
       <c r="I62">
-        <v>5.042608499526978</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -4872,7 +4872,7 @@
         <v>1</v>
       </c>
       <c r="I63">
-        <v>3.280902147293091</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64" spans="1:9">
@@ -4901,7 +4901,7 @@
         <v>0</v>
       </c>
       <c r="I64">
-        <v>4.683549404144287</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -4930,7 +4930,7 @@
         <v>1</v>
       </c>
       <c r="I65">
-        <v>5.288894891738892</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66" spans="1:9">
@@ -4959,7 +4959,7 @@
         <v>1</v>
       </c>
       <c r="I66">
-        <v>6.951707124710083</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67" spans="1:9">
@@ -4988,7 +4988,7 @@
         <v>0</v>
       </c>
       <c r="I67">
-        <v>3.770574569702148</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68" spans="1:9">
@@ -5014,7 +5014,7 @@
         <v>0</v>
       </c>
       <c r="I68">
-        <v>26.57816290855408</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -5043,7 +5043,7 @@
         <v>0</v>
       </c>
       <c r="I69">
-        <v>6.570940017700195</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -5072,7 +5072,7 @@
         <v>1</v>
       </c>
       <c r="I70">
-        <v>5.117671251296997</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:9">
@@ -5101,7 +5101,7 @@
         <v>1</v>
       </c>
       <c r="I71">
-        <v>4.607646942138672</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72" spans="1:9">
@@ -5130,7 +5130,7 @@
         <v>1</v>
       </c>
       <c r="I72">
-        <v>6.901288509368896</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73" spans="1:9">
@@ -5159,7 +5159,7 @@
         <v>0</v>
       </c>
       <c r="I73">
-        <v>5.888517618179321</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:9">
@@ -5188,7 +5188,7 @@
         <v>0</v>
       </c>
       <c r="I74">
-        <v>3.694136619567871</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75" spans="1:9">
@@ -5217,7 +5217,7 @@
         <v>0</v>
       </c>
       <c r="I75">
-        <v>3.997627973556519</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -5246,7 +5246,7 @@
         <v>0</v>
       </c>
       <c r="I76">
-        <v>3.38338303565979</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -5275,7 +5275,7 @@
         <v>0</v>
       </c>
       <c r="I77">
-        <v>4.824132919311523</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78" spans="1:9">
@@ -5304,7 +5304,7 @@
         <v>1</v>
       </c>
       <c r="I78">
-        <v>2.88294506072998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79" spans="1:9">
@@ -5333,7 +5333,7 @@
         <v>0</v>
       </c>
       <c r="I79">
-        <v>5.969459772109985</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80" spans="1:9">
@@ -5362,7 +5362,7 @@
         <v>0</v>
       </c>
       <c r="I80">
-        <v>4.981320142745972</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81" spans="1:9">
@@ -5391,7 +5391,7 @@
         <v>0</v>
       </c>
       <c r="I81">
-        <v>4.081705808639526</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82" spans="1:9">
@@ -5420,7 +5420,7 @@
         <v>0</v>
       </c>
       <c r="I82">
-        <v>11.17678093910217</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83" spans="1:9">
@@ -5449,7 +5449,7 @@
         <v>1</v>
       </c>
       <c r="I83">
-        <v>7.056002140045166</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84" spans="1:9">
@@ -5478,7 +5478,7 @@
         <v>0</v>
       </c>
       <c r="I84">
-        <v>6.249098539352417</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85" spans="1:9">
@@ -5507,7 +5507,7 @@
         <v>0</v>
       </c>
       <c r="I85">
-        <v>7.374261856079102</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86" spans="1:9">
@@ -5536,7 +5536,7 @@
         <v>0</v>
       </c>
       <c r="I86">
-        <v>8.768988847732544</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87" spans="1:9">
@@ -5565,7 +5565,7 @@
         <v>1</v>
       </c>
       <c r="I87">
-        <v>9.570739269256592</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88" spans="1:9">
@@ -5594,7 +5594,7 @@
         <v>1</v>
       </c>
       <c r="I88">
-        <v>7.524593830108643</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89" spans="1:9">
@@ -5623,7 +5623,7 @@
         <v>0</v>
       </c>
       <c r="I89">
-        <v>5.225824117660522</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90" spans="1:9">
@@ -5652,7 +5652,7 @@
         <v>1</v>
       </c>
       <c r="I90">
-        <v>5.344269275665283</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91" spans="1:9">
@@ -5681,7 +5681,7 @@
         <v>0</v>
       </c>
       <c r="I91">
-        <v>7.093771934509277</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92" spans="1:9">
@@ -5710,7 +5710,7 @@
         <v>0</v>
       </c>
       <c r="I92">
-        <v>8.500173330307007</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93" spans="1:9">
@@ -5739,7 +5739,7 @@
         <v>0</v>
       </c>
       <c r="I93">
-        <v>6.901445627212524</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94" spans="1:9">
@@ -5768,7 +5768,7 @@
         <v>0</v>
       </c>
       <c r="I94">
-        <v>4.815563440322876</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95" spans="1:9">
@@ -5797,7 +5797,7 @@
         <v>1</v>
       </c>
       <c r="I95">
-        <v>7.250130891799927</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96" spans="1:9">
@@ -5826,7 +5826,7 @@
         <v>0</v>
       </c>
       <c r="I96">
-        <v>4.826891422271729</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97" spans="1:9">
@@ -5855,7 +5855,7 @@
         <v>1</v>
       </c>
       <c r="I97">
-        <v>5.017213821411133</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98" spans="1:9">
@@ -5884,7 +5884,7 @@
         <v>0</v>
       </c>
       <c r="I98">
-        <v>6.053272008895874</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99" spans="1:9">
@@ -5913,7 +5913,7 @@
         <v>0</v>
       </c>
       <c r="I99">
-        <v>26.78950166702271</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100" spans="1:9">
@@ -5942,7 +5942,7 @@
         <v>0</v>
       </c>
       <c r="I100">
-        <v>5.897969007492065</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101" spans="1:9">
@@ -5971,7 +5971,7 @@
         <v>0</v>
       </c>
       <c r="I101">
-        <v>5.797082901000977</v>
+        <v>0</v>
       </c>
     </row>
     <row r="102" spans="1:9">
@@ -6000,7 +6000,7 @@
         <v>0</v>
       </c>
       <c r="I102">
-        <v>5.689821481704712</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103" spans="1:9">
@@ -6029,7 +6029,7 @@
         <v>0</v>
       </c>
       <c r="I103">
-        <v>4.501355409622192</v>
+        <v>0</v>
       </c>
     </row>
     <row r="104" spans="1:9">
@@ -6058,7 +6058,7 @@
         <v>1</v>
       </c>
       <c r="I104">
-        <v>7.329994201660156</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105" spans="1:9">
@@ -6087,7 +6087,7 @@
         <v>0</v>
       </c>
       <c r="I105">
-        <v>5.640607118606567</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106" spans="1:9">
@@ -6116,7 +6116,7 @@
         <v>0</v>
       </c>
       <c r="I106">
-        <v>5.33793306350708</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107" spans="1:9">
@@ -6145,7 +6145,7 @@
         <v>0</v>
       </c>
       <c r="I107">
-        <v>11.87717366218567</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108" spans="1:9">
@@ -6174,7 +6174,7 @@
         <v>0</v>
       </c>
       <c r="I108">
-        <v>7.986060857772827</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:9">
@@ -6203,7 +6203,7 @@
         <v>1</v>
       </c>
       <c r="I109">
-        <v>5.527501821517944</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:9">
@@ -6232,7 +6232,7 @@
         <v>1</v>
       </c>
       <c r="I110">
-        <v>9.815976858139038</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111" spans="1:9">
@@ -6261,7 +6261,7 @@
         <v>0</v>
       </c>
       <c r="I111">
-        <v>8.207018613815308</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112" spans="1:9">
@@ -6290,7 +6290,7 @@
         <v>1</v>
       </c>
       <c r="I112">
-        <v>7.756214141845703</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113" spans="1:9">
@@ -6319,7 +6319,7 @@
         <v>1</v>
       </c>
       <c r="I113">
-        <v>4.240583419799805</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114" spans="1:9">
@@ -6348,7 +6348,7 @@
         <v>0</v>
       </c>
       <c r="I114">
-        <v>6.076520204544067</v>
+        <v>0</v>
       </c>
     </row>
     <row r="115" spans="1:9">
@@ -6377,7 +6377,7 @@
         <v>0</v>
       </c>
       <c r="I115">
-        <v>7.885587453842163</v>
+        <v>0</v>
       </c>
     </row>
     <row r="116" spans="1:9">
@@ -6406,7 +6406,7 @@
         <v>0</v>
       </c>
       <c r="I116">
-        <v>5.587735414505005</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117" spans="1:9">
@@ -6435,7 +6435,7 @@
         <v>0</v>
       </c>
       <c r="I117">
-        <v>4.166070699691772</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118" spans="1:9">
@@ -6464,7 +6464,7 @@
         <v>0</v>
       </c>
       <c r="I118">
-        <v>4.905081033706665</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119" spans="1:9">
@@ -6493,7 +6493,7 @@
         <v>1</v>
       </c>
       <c r="I119">
-        <v>9.90749979019165</v>
+        <v>0</v>
       </c>
     </row>
     <row r="120" spans="1:9">
@@ -6522,7 +6522,7 @@
         <v>1</v>
       </c>
       <c r="I120">
-        <v>10.56476283073425</v>
+        <v>0</v>
       </c>
     </row>
     <row r="121" spans="1:9">
@@ -6551,7 +6551,7 @@
         <v>1</v>
       </c>
       <c r="I121">
-        <v>32.30186605453491</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>